<commit_message>
Update World Cup prediction pages
</commit_message>
<xml_diff>
--- a/2026世界杯淘汰赛赛程表_中文版_Codex.xlsx
+++ b/2026世界杯淘汰赛赛程表_中文版_Codex.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰赛赛程" sheetId="1" r:id="Rc19f7c2af3094548"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rd1820597e5aa4ee6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰赛赛程" sheetId="1" r:id="R3264bd1d10cd4b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R96565f4df969448d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -183,9 +183,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1587,19 +1587,23 @@
         <x:v>16强赛</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>待定：53452545胜者</x:v>
+        <x:v>加拿大</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>TBD: Winner of 53452545</x:v>
-      </x:c>
-      <x:c r="G18" s="14" t="str"/>
+        <x:v>Canada</x:v>
+      </x:c>
+      <x:c r="G18" s="14" t="str">
+        <x:v>CAN</x:v>
+      </x:c>
       <x:c r="H18" s="14" t="str">
-        <x:v>待定：53452547胜者</x:v>
+        <x:v>荷兰</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
-        <x:v>TBD: Winner of 53452547</x:v>
-      </x:c>
-      <x:c r="J18" s="14" t="str"/>
+        <x:v>Netherlands</x:v>
+      </x:c>
+      <x:c r="J18" s="14" t="str">
+        <x:v>NED</x:v>
+      </x:c>
       <x:c r="K18" s="14" t="str">
         <x:v>2026-07-04 13:00:00 -04:00</x:v>
       </x:c>
@@ -1657,19 +1661,23 @@
         <x:v>16强赛</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>待定：53452541胜者</x:v>
+        <x:v>德国</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>TBD: Winner of 53452541</x:v>
-      </x:c>
-      <x:c r="G19" s="14" t="str"/>
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="G19" s="14" t="str">
+        <x:v>GER</x:v>
+      </x:c>
       <x:c r="H19" s="14" t="str">
-        <x:v>待定：53452543胜者</x:v>
+        <x:v>法国</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>TBD: Winner of 53452543</x:v>
-      </x:c>
-      <x:c r="J19" s="14" t="str"/>
+        <x:v>France</x:v>
+      </x:c>
+      <x:c r="J19" s="14" t="str">
+        <x:v>FRA</x:v>
+      </x:c>
       <x:c r="K19" s="14" t="str">
         <x:v>2026-07-04 17:00:00 -04:00</x:v>
       </x:c>
@@ -1727,19 +1735,23 @@
         <x:v>16强赛</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
-        <x:v>待定：53452557胜者</x:v>
+        <x:v>巴西</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>TBD: Winner of 53452557</x:v>
-      </x:c>
-      <x:c r="G20" s="14" t="str"/>
+        <x:v>Brazil</x:v>
+      </x:c>
+      <x:c r="G20" s="14" t="str">
+        <x:v>BRA</x:v>
+      </x:c>
       <x:c r="H20" s="14" t="str">
-        <x:v>待定：53452561胜者</x:v>
+        <x:v>挪威</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
-        <x:v>TBD: Winner of 53452561</x:v>
-      </x:c>
-      <x:c r="J20" s="14" t="str"/>
+        <x:v>Norway</x:v>
+      </x:c>
+      <x:c r="J20" s="14" t="str">
+        <x:v>NOR</x:v>
+      </x:c>
       <x:c r="K20" s="14" t="str">
         <x:v>2026-07-05 16:00:00 -04:00</x:v>
       </x:c>
@@ -1797,19 +1809,23 @@
         <x:v>16强赛</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>待定：53452563胜者</x:v>
+        <x:v>墨西哥</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>TBD: Winner of 53452563</x:v>
-      </x:c>
-      <x:c r="G21" s="14" t="str"/>
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="G21" s="14" t="str">
+        <x:v>MEX</x:v>
+      </x:c>
       <x:c r="H21" s="14" t="str">
-        <x:v>待定：53452565胜者</x:v>
+        <x:v>英格兰</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>TBD: Winner of 53452565</x:v>
-      </x:c>
-      <x:c r="J21" s="14" t="str"/>
+        <x:v>England</x:v>
+      </x:c>
+      <x:c r="J21" s="14" t="str">
+        <x:v>ENG</x:v>
+      </x:c>
       <x:c r="K21" s="14" t="str">
         <x:v>2026-07-05 20:00:00 -04:00</x:v>
       </x:c>
@@ -1867,19 +1883,23 @@
         <x:v>16强赛</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>待定：53452549胜者</x:v>
+        <x:v>葡萄牙</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>TBD: Winner of 53452549</x:v>
-      </x:c>
-      <x:c r="G22" s="14" t="str"/>
+        <x:v>Portugal</x:v>
+      </x:c>
+      <x:c r="G22" s="14" t="str">
+        <x:v>POR</x:v>
+      </x:c>
       <x:c r="H22" s="14" t="str">
-        <x:v>待定：53452551胜者</x:v>
+        <x:v>西班牙</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>TBD: Winner of 53452551</x:v>
-      </x:c>
-      <x:c r="J22" s="14" t="str"/>
+        <x:v>Spain</x:v>
+      </x:c>
+      <x:c r="J22" s="14" t="str">
+        <x:v>ESP</x:v>
+      </x:c>
       <x:c r="K22" s="14" t="str">
         <x:v>2026-07-06 15:00:00 -04:00</x:v>
       </x:c>
@@ -1937,19 +1957,23 @@
         <x:v>16强赛</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>待定：53452553胜者</x:v>
+        <x:v>美国</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>TBD: Winner of 53452553</x:v>
-      </x:c>
-      <x:c r="G23" s="14" t="str"/>
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="G23" s="14" t="str">
+        <x:v>USA</x:v>
+      </x:c>
       <x:c r="H23" s="14" t="str">
-        <x:v>待定：53452555胜者</x:v>
+        <x:v>比利时</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>TBD: Winner of 53452555</x:v>
-      </x:c>
-      <x:c r="J23" s="14" t="str"/>
+        <x:v>Belgium</x:v>
+      </x:c>
+      <x:c r="J23" s="14" t="str">
+        <x:v>BEL</x:v>
+      </x:c>
       <x:c r="K23" s="14" t="str">
         <x:v>2026-07-06 20:00:00 -04:00</x:v>
       </x:c>
@@ -2077,19 +2101,21 @@
         <x:v>16强赛</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
-        <x:v>待定：53452505胜者</x:v>
+        <x:v>瑞士</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>TBD: Winner of 53452505</x:v>
-      </x:c>
-      <x:c r="G25" s="14" t="str"/>
+        <x:v>Switzerland</x:v>
+      </x:c>
+      <x:c r="G25" s="14" t="str">
+        <x:v>SUI</x:v>
+      </x:c>
       <x:c r="H25" s="14" t="str">
         <x:v>待定：53452507胜者</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
         <x:v>TBD: Winner of 53452507</x:v>
       </x:c>
-      <x:c r="J25" s="14" t="str"/>
+      <x:c r="J25" s="14"/>
       <x:c r="K25" s="14" t="str">
         <x:v>2026-07-07 16:00:00 -04:00</x:v>
       </x:c>
@@ -2692,7 +2718,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R574c294ebe2f4da9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99ae33fd81154bb2"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>